<commit_message>
Rebuild tm grid as one best-selling model per 5-tm class; add single review slide
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Pbxjp9hvsGyGE8VjiFxi6d
</commit_message>
<xml_diff>
--- a/analysis/Pareto_tm_Class.xlsx
+++ b/analysis/Pareto_tm_Class.xlsx
@@ -20,7 +20,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;Rp &quot;#,##0"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -51,6 +51,11 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="005A6570"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="5">
@@ -102,7 +107,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -117,20 +122,21 @@
     <xf numFmtId="9" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2311,31 +2317,33 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
     <col width="24" customWidth="1" min="7" max="7"/>
     <col width="24" customWidth="1" min="8" max="8"/>
-    <col width="48" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Medium class: popular models (Pareto top 5 by units or value) by Max Lifting Moment, Jan 2023 – 14 Aug 2026</t>
+          <t>Medium class: best-selling model in each 5-tm class vs F.lli Ferrari, Jan 2023 – 14 Aug 2026</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cell = model (tm) · units · import value. Ferrari = models in the 2026 catalogue; price = TSP price list, crane only, incl. tax.</t>
+          <t>Cell = model (tm) · units · share of class units · price per unit, crane only (IDR, incl. tax). Best seller = most units in the class (variants merged).</t>
         </is>
       </c>
     </row>
@@ -2357,36 +2365,16 @@
       </c>
       <c r="D3" s="11" t="inlineStr">
         <is>
-          <t>Palfinger</t>
-        </is>
-      </c>
-      <c r="E3" s="11" t="inlineStr">
-        <is>
-          <t>XCMG</t>
-        </is>
-      </c>
-      <c r="F3" s="11" t="inlineStr">
-        <is>
           <t>Amco Veba</t>
         </is>
       </c>
-      <c r="G3" s="11" t="inlineStr">
-        <is>
-          <t>Hiab</t>
-        </is>
-      </c>
-      <c r="H3" s="11" t="inlineStr">
-        <is>
-          <t>Hyva</t>
-        </is>
-      </c>
-      <c r="I3" s="12" t="inlineStr">
+      <c r="E3" s="12" t="inlineStr">
         <is>
           <t>F.lli Ferrari</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="45" customHeight="1">
+    <row r="4" ht="48" customHeight="1">
       <c r="A4" s="13" t="inlineStr">
         <is>
           <t>&gt;25–30</t>
@@ -2395,25 +2383,21 @@
       <c r="B4" s="14" t="n">
         <v>49</v>
       </c>
-      <c r="C4" s="14" t="inlineStr"/>
-      <c r="D4" s="14" t="inlineStr"/>
-      <c r="E4" s="14" t="inlineStr"/>
-      <c r="F4" s="14" t="inlineStr">
-        <is>
-          <t>V825 (25.6) · 31 units · Rp 16.030.000.000</t>
-        </is>
-      </c>
-      <c r="G4" s="14" t="inlineStr"/>
-      <c r="H4" s="14" t="inlineStr"/>
-      <c r="I4" s="15" t="inlineStr">
-        <is>
-          <t>730 (27.4) · price not yet known
-268 (25.4) · 268 A3: Rp 620.000.000 / 268 A4: Rp 670.000.000
-FST 12 (30) · price not yet known</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="120" customHeight="1">
+      <c r="C4" s="14" t="n"/>
+      <c r="D4" s="13" t="inlineStr">
+        <is>
+          <t>V825 (25.6 tm)
+31 units · 63% of class
+Rp 620.000.000 per unit</t>
+        </is>
+      </c>
+      <c r="E4" s="15" t="inlineStr">
+        <is>
+          <t>268 A4 (25.4 tm) · Rp 670.000.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="48" customHeight="1">
       <c r="A5" s="13" t="inlineStr">
         <is>
           <t>&gt;30–35</t>
@@ -2422,34 +2406,21 @@
       <c r="B5" s="14" t="n">
         <v>77</v>
       </c>
-      <c r="C5" s="14" t="inlineStr">
-        <is>
-          <t>SPK32080 (30.4) · 33 units · Rp 12.860.000.000</t>
-        </is>
-      </c>
-      <c r="D5" s="14" t="inlineStr"/>
-      <c r="E5" s="14" t="inlineStr"/>
-      <c r="F5" s="14" t="inlineStr"/>
-      <c r="G5" s="14" t="inlineStr">
-        <is>
-          <t>X-CLX 388 (34.3) · 21 units · Rp 16.000.000.000</t>
-        </is>
-      </c>
-      <c r="H5" s="14" t="inlineStr"/>
-      <c r="I5" s="15" t="inlineStr">
-        <is>
-          <t>7401C (34.8) · price not yet known
-7401SC (32.9) · price not yet known
-734 (30.3) · price not yet known
-738R (31.3) · price not yet known
-9405C (34.8) · price not yet known
-FBR 330 (31.8) · price not yet known
-FBR 350 (32.8) · FBR350 A4: Rp 1.250.000.000 / FBR350R A4: Rp 1.440.000.000
-FST 14 (35) · price not yet known</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="30" customHeight="1">
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>SPK32080 (30.4 tm)
+33 units · 43% of class
+Rp 440.000.000 per unit</t>
+        </is>
+      </c>
+      <c r="D5" s="14" t="n"/>
+      <c r="E5" s="15" t="inlineStr">
+        <is>
+          <t>FBR350R A4 (32.8 tm) · Rp 1.440.000.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="48" customHeight="1">
       <c r="A6" s="13" t="inlineStr">
         <is>
           <t>&gt;35–40</t>
@@ -2458,28 +2429,21 @@
       <c r="B6" s="14" t="n">
         <v>66</v>
       </c>
-      <c r="C6" s="14" t="inlineStr">
-        <is>
-          <t>SPK36080 (36) · 34 units · Rp 14.710.000.000</t>
-        </is>
-      </c>
-      <c r="D6" s="14" t="inlineStr">
-        <is>
-          <t>PK 41002 (38.4) · 21 units · Rp 23.170.000.000</t>
-        </is>
-      </c>
-      <c r="E6" s="14" t="inlineStr"/>
-      <c r="F6" s="14" t="inlineStr"/>
-      <c r="G6" s="14" t="inlineStr"/>
-      <c r="H6" s="14" t="inlineStr"/>
-      <c r="I6" s="15" t="inlineStr">
-        <is>
-          <t>7441C (37.7) · price not yet known
-9445C (37.7) · price not yet known</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
+      <c r="C6" s="13" t="inlineStr">
+        <is>
+          <t>SPK36080 (36 tm)
+34 units · 52% of class
+Rp 490.000.000 per unit</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="n"/>
+      <c r="E6" s="15" t="inlineStr">
+        <is>
+          <t>7441C (37.7 tm) · price not yet known</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="48" customHeight="1">
       <c r="A7" s="13" t="inlineStr">
         <is>
           <t>&gt;40–45</t>
@@ -2488,30 +2452,31 @@
       <c r="B7" s="14" t="n">
         <v>26</v>
       </c>
-      <c r="C7" s="14" t="inlineStr"/>
-      <c r="D7" s="14" t="inlineStr"/>
-      <c r="E7" s="14" t="inlineStr"/>
-      <c r="F7" s="14" t="inlineStr"/>
-      <c r="G7" s="14" t="inlineStr"/>
-      <c r="H7" s="14" t="inlineStr"/>
-      <c r="I7" s="15" t="inlineStr">
-        <is>
-          <t>746R (43.4) · 746 A4: Rp 1.860.000.000
-749R (44.7) · 749R A4: Rp 2.210.000.000</t>
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>SPK42502 (42.5 tm)
+18 units · 69% of class
+Rp 790.000.000 per unit</t>
+        </is>
+      </c>
+      <c r="D7" s="14" t="n"/>
+      <c r="E7" s="15" t="inlineStr">
+        <is>
+          <t>746 A4 (43.4 tm) · Rp 1.860.000.000</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
         <is>
-          <t>Heavy class: popular models (Pareto top 5 by units or value) by Max Lifting Moment, Jan 2023 – 14 Aug 2026</t>
+          <t>Heavy class: best-selling model in each 5-tm class vs F.lli Ferrari, Jan 2023 – 14 Aug 2026</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Cell = model (tm) · units · import value. Ferrari = models in the 2026 catalogue; price = TSP price list, crane only, incl. tax.</t>
+          <t>Cell = model (tm) · units · share of class units · price per unit, crane only (IDR, incl. tax). Best seller = most units in the class (variants merged).</t>
         </is>
       </c>
     </row>
@@ -2548,21 +2513,16 @@
       </c>
       <c r="G12" s="11" t="inlineStr">
         <is>
-          <t>Hiab</t>
-        </is>
-      </c>
-      <c r="H12" s="11" t="inlineStr">
-        <is>
           <t>Hyva</t>
         </is>
       </c>
-      <c r="I12" s="12" t="inlineStr">
+      <c r="H12" s="12" t="inlineStr">
         <is>
           <t>F.lli Ferrari</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="45" customHeight="1">
+    <row r="13" ht="48" customHeight="1">
       <c r="A13" s="13" t="inlineStr">
         <is>
           <t>&gt;45–50</t>
@@ -2571,33 +2531,24 @@
       <c r="B13" s="14" t="n">
         <v>22</v>
       </c>
-      <c r="C13" s="14" t="inlineStr"/>
-      <c r="D13" s="14" t="inlineStr"/>
-      <c r="E13" s="14" t="inlineStr">
-        <is>
-          <t>GSQZ460.4 (46) · 3 units · Rp 2.150.000.000</t>
-        </is>
-      </c>
-      <c r="F13" s="14" t="inlineStr">
-        <is>
-          <t>V950 (45.9) · 12 units · Rp 18.900.000.000</t>
-        </is>
-      </c>
-      <c r="G13" s="14" t="inlineStr"/>
-      <c r="H13" s="14" t="inlineStr">
-        <is>
-          <t>HC501X (50) · 4 units · Rp 4.280.000.000</t>
-        </is>
-      </c>
-      <c r="I13" s="15" t="inlineStr">
-        <is>
-          <t>745 (45.1) · price not yet known
-FBR 450 (45.5) · FBR450 A4: Rp 1.580.000.000 / FBR450R A4: Rp 1.780.000.000 / FBR450R A6: Rp 1.880.000.000
-FVT 455 (45.7) · price not yet known</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="18" customHeight="1">
+      <c r="C13" s="14" t="n"/>
+      <c r="D13" s="14" t="n"/>
+      <c r="E13" s="14" t="n"/>
+      <c r="F13" s="13" t="inlineStr">
+        <is>
+          <t>V950 (45.9 tm)
+12 units · 55% of class
+Rp 1.880.000.000 per unit</t>
+        </is>
+      </c>
+      <c r="G13" s="14" t="n"/>
+      <c r="H13" s="15" t="inlineStr">
+        <is>
+          <t>FBR450R A4 (45.5 tm) · Rp 1.780.000.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="48" customHeight="1">
       <c r="A14" s="13" t="inlineStr">
         <is>
           <t>&gt;50–55</t>
@@ -2606,23 +2557,24 @@
       <c r="B14" s="14" t="n">
         <v>40</v>
       </c>
-      <c r="C14" s="14" t="inlineStr"/>
-      <c r="D14" s="14" t="inlineStr">
-        <is>
-          <t>PK 53002 (50.1) · 39 units · Rp 53.080.000.000</t>
-        </is>
-      </c>
-      <c r="E14" s="14" t="inlineStr"/>
-      <c r="F14" s="14" t="inlineStr"/>
-      <c r="G14" s="14" t="inlineStr"/>
-      <c r="H14" s="14" t="inlineStr"/>
-      <c r="I14" s="15" t="inlineStr">
+      <c r="C14" s="14" t="n"/>
+      <c r="D14" s="13" t="inlineStr">
+        <is>
+          <t>PK 53002 (50.1 tm)
+39 units · 98% of class
+Rp 1.620.000.000 per unit</t>
+        </is>
+      </c>
+      <c r="E14" s="14" t="n"/>
+      <c r="F14" s="14" t="n"/>
+      <c r="G14" s="14" t="n"/>
+      <c r="H14" s="15" t="inlineStr">
         <is>
           <t>No Ferrari model</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="45" customHeight="1">
+    <row r="15" ht="48" customHeight="1">
       <c r="A15" s="13" t="inlineStr">
         <is>
           <t>&gt;55–60</t>
@@ -2631,25 +2583,24 @@
       <c r="B15" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="C15" s="14" t="inlineStr"/>
-      <c r="D15" s="14" t="inlineStr"/>
-      <c r="E15" s="14" t="inlineStr"/>
-      <c r="F15" s="14" t="inlineStr"/>
-      <c r="G15" s="14" t="inlineStr"/>
-      <c r="H15" s="14" t="inlineStr">
-        <is>
-          <t>HB660R (60) · 2 units · Rp 3.090.000.000</t>
-        </is>
-      </c>
-      <c r="I15" s="15" t="inlineStr">
-        <is>
-          <t>9601C (57.5) · price not yet known
-FBR 600 (57.4) · FBR600R A4: Rp 2.620.000.000
-FBR 660 (58.8) · FBR660R A4: Rp 2.660.000.000 / FBR660R A6: Rp 2.840.000.000</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="18" customHeight="1">
+      <c r="C15" s="14" t="n"/>
+      <c r="D15" s="14" t="n"/>
+      <c r="E15" s="14" t="n"/>
+      <c r="F15" s="14" t="n"/>
+      <c r="G15" s="13" t="inlineStr">
+        <is>
+          <t>HB660R (60 tm)
+2 units · 67% of class
+Rp 1.840.000.000 per unit</t>
+        </is>
+      </c>
+      <c r="H15" s="15" t="inlineStr">
+        <is>
+          <t>FBR660R A4 (58.8 tm) · Rp 2.660.000.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="48" customHeight="1">
       <c r="A16" s="13" t="inlineStr">
         <is>
           <t>&gt;60–65</t>
@@ -2658,19 +2609,24 @@
       <c r="B16" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="C16" s="14" t="inlineStr"/>
-      <c r="D16" s="14" t="inlineStr"/>
-      <c r="E16" s="14" t="inlineStr"/>
-      <c r="F16" s="14" t="inlineStr"/>
-      <c r="G16" s="14" t="inlineStr"/>
-      <c r="H16" s="14" t="inlineStr"/>
-      <c r="I16" s="15" t="inlineStr">
-        <is>
-          <t>9661C (63.2) · price not yet known</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="18" customHeight="1">
+      <c r="C16" s="13" t="inlineStr">
+        <is>
+          <t>SPK61502 (61.5 tm)
+1 units · 100% of class
+Rp 1.400.000.000 per unit</t>
+        </is>
+      </c>
+      <c r="D16" s="14" t="n"/>
+      <c r="E16" s="14" t="n"/>
+      <c r="F16" s="14" t="n"/>
+      <c r="G16" s="14" t="n"/>
+      <c r="H16" s="15" t="inlineStr">
+        <is>
+          <t>9661C (63.2 tm) · price not yet known</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="48" customHeight="1">
       <c r="A17" s="13" t="inlineStr">
         <is>
           <t>&gt;70–75</t>
@@ -2679,23 +2635,24 @@
       <c r="B17" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="C17" s="14" t="inlineStr"/>
-      <c r="D17" s="14" t="inlineStr">
-        <is>
-          <t>PK 76002 EH D (71.6) · 2 units · Rp 3.840.000.000</t>
-        </is>
-      </c>
-      <c r="E17" s="14" t="inlineStr"/>
-      <c r="F17" s="14" t="inlineStr"/>
-      <c r="G17" s="14" t="inlineStr"/>
-      <c r="H17" s="14" t="inlineStr"/>
-      <c r="I17" s="15" t="inlineStr">
-        <is>
-          <t>990R (74) · price not yet known</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="18" customHeight="1">
+      <c r="C17" s="14" t="n"/>
+      <c r="D17" s="13" t="inlineStr">
+        <is>
+          <t>PK 76002 EH D (71.6 tm)
+2 units · 100% of class
+Rp 2.290.000.000 per unit</t>
+        </is>
+      </c>
+      <c r="E17" s="14" t="n"/>
+      <c r="F17" s="14" t="n"/>
+      <c r="G17" s="14" t="n"/>
+      <c r="H17" s="15" t="inlineStr">
+        <is>
+          <t>990R (74 tm) · price not yet known</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="48" customHeight="1">
       <c r="A18" s="13" t="inlineStr">
         <is>
           <t>&gt;80–85</t>
@@ -2704,19 +2661,24 @@
       <c r="B18" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="C18" s="14" t="inlineStr"/>
-      <c r="D18" s="14" t="inlineStr"/>
-      <c r="E18" s="14" t="inlineStr"/>
-      <c r="F18" s="14" t="inlineStr"/>
-      <c r="G18" s="14" t="inlineStr"/>
-      <c r="H18" s="14" t="inlineStr"/>
-      <c r="I18" s="15" t="inlineStr">
+      <c r="C18" s="14" t="n"/>
+      <c r="D18" s="13" t="inlineStr">
+        <is>
+          <t>PK 88002 EH C (81.6 tm)
+1 units · 100% of class
+Rp 2.220.000.000 per unit</t>
+        </is>
+      </c>
+      <c r="E18" s="14" t="n"/>
+      <c r="F18" s="14" t="n"/>
+      <c r="G18" s="14" t="n"/>
+      <c r="H18" s="15" t="inlineStr">
         <is>
           <t>No Ferrari model</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="18" customHeight="1">
+    <row r="19" ht="48" customHeight="1">
       <c r="A19" s="13" t="inlineStr">
         <is>
           <t>&gt;85–90</t>
@@ -2725,15 +2687,34 @@
       <c r="B19" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="C19" s="14" t="inlineStr"/>
-      <c r="D19" s="14" t="inlineStr"/>
-      <c r="E19" s="14" t="inlineStr"/>
-      <c r="F19" s="14" t="inlineStr"/>
-      <c r="G19" s="14" t="inlineStr"/>
-      <c r="H19" s="14" t="inlineStr"/>
-      <c r="I19" s="15" t="inlineStr">
+      <c r="C19" s="14" t="n"/>
+      <c r="D19" s="14" t="n"/>
+      <c r="E19" s="13" t="inlineStr">
+        <is>
+          <t>GSQZ880.6 (88 tm)
+2 units · 50% of class
+Rp 1.320.000.000 per unit</t>
+        </is>
+      </c>
+      <c r="F19" s="14" t="n"/>
+      <c r="G19" s="14" t="n"/>
+      <c r="H19" s="15" t="inlineStr">
         <is>
           <t>No Ferrari model</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="16" t="inlineStr">
+        <is>
+          <t>Competitor price = average import unit price 2023–2026 × Rp 17.803/USD (JISDOR 23 Sep 2026) × (1 + import duty: 0% China – ACFTA, 5% Europe – assumed) × (1 + PPN 11% + PPh 22 2.5%). Import cost before distributor margin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="16" t="inlineStr">
+        <is>
+          <t>Ferrari price = TSP selling price to customers, crane only, incl. GP, warranty and tax (price list). Ferrari model = the priced catalogue model closest in tm to the best seller. Prices rounded to Rp 10.000.000.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Exclude Hyva; add product photos to tm positioning slides
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Pbxjp9hvsGyGE8VjiFxi6d
</commit_message>
<xml_diff>
--- a/analysis/Pareto_tm_Class.xlsx
+++ b/analysis/Pareto_tm_Class.xlsx
@@ -1263,7 +1263,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Top 5 = 64% of class units; 8 of 27 models reach 80%. Variants merged (e.g. SPK32080/B/C, PK 41002 EH C/MH C).</t>
+          <t>Top 5 = 65% of class units; 7 of 24 models reach 80%. Variants merged (e.g. SPK32080/B/C, PK 41002 EH C/MH C).</t>
         </is>
       </c>
     </row>
@@ -1343,10 +1343,10 @@
         <v>14710000000</v>
       </c>
       <c r="H4" s="6" t="n">
-        <v>0.1559633027522936</v>
+        <v>0.1588785046728972</v>
       </c>
       <c r="I4" s="6" t="n">
-        <v>0.1559633027522936</v>
+        <v>0.1588785046728972</v>
       </c>
     </row>
     <row r="5">
@@ -1378,10 +1378,10 @@
         <v>12860000000</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>0.1513761467889908</v>
+        <v>0.1542056074766355</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>0.3073394495412844</v>
+        <v>0.3130841121495327</v>
       </c>
     </row>
     <row r="6">
@@ -1413,10 +1413,10 @@
         <v>16030000000</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>0.1422018348623853</v>
+        <v>0.1448598130841121</v>
       </c>
       <c r="I6" s="6" t="n">
-        <v>0.4495412844036698</v>
+        <v>0.4579439252336448</v>
       </c>
     </row>
     <row r="7">
@@ -1448,10 +1448,10 @@
         <v>23170000000</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>0.0963302752293578</v>
+        <v>0.09813084112149532</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>0.5458715596330276</v>
+        <v>0.5560747663551401</v>
       </c>
     </row>
     <row r="8">
@@ -1483,10 +1483,10 @@
         <v>16000000000</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>0.0963302752293578</v>
+        <v>0.09813084112149532</v>
       </c>
       <c r="I8" s="6" t="n">
-        <v>0.6422018348623854</v>
+        <v>0.6542056074766354</v>
       </c>
     </row>
     <row r="9">
@@ -1498,19 +1498,19 @@
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>22 models</t>
+          <t>19 models</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr"/>
       <c r="E9" s="7" t="inlineStr"/>
       <c r="F9" s="7" t="n">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="G9" s="8" t="n">
-        <v>47270000000</v>
+        <v>43750000000</v>
       </c>
       <c r="H9" s="9" t="n">
-        <v>0.3577981651376145</v>
+        <v>0.3457943925233645</v>
       </c>
       <c r="I9" s="9" t="n">
         <v>1</v>
@@ -1526,7 +1526,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Top 5 = 64% of class import value; 8 of 27 models reach 80%. Variants merged (e.g. SPK32080/B/C, PK 41002 EH C/MH C).</t>
+          <t>Top 5 = 65% of class import value; 7 of 24 models reach 80%. Variants merged (e.g. SPK32080/B/C, PK 41002 EH C/MH C).</t>
         </is>
       </c>
     </row>
@@ -1606,10 +1606,10 @@
         <v>23170000000</v>
       </c>
       <c r="H18" s="6" t="n">
-        <v>0.1781378926107584</v>
+        <v>0.1830937462443117</v>
       </c>
       <c r="I18" s="6" t="n">
-        <v>0.1781378926107584</v>
+        <v>0.1830937462443117</v>
       </c>
     </row>
     <row r="19">
@@ -1641,10 +1641,10 @@
         <v>16030000000</v>
       </c>
       <c r="H19" s="6" t="n">
-        <v>0.1232831034669731</v>
+        <v>0.1267128791722888</v>
       </c>
       <c r="I19" s="6" t="n">
-        <v>0.3014209960777315</v>
+        <v>0.3098066254166004</v>
       </c>
     </row>
     <row r="20">
@@ -1676,10 +1676,10 @@
         <v>16000000000</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>0.1230744369779903</v>
+        <v>0.1264984075142739</v>
       </c>
       <c r="I20" s="6" t="n">
-        <v>0.4244954330557218</v>
+        <v>0.4363050329308743</v>
       </c>
     </row>
     <row r="21">
@@ -1711,10 +1711,10 @@
         <v>14710000000</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>0.1130868255402569</v>
+        <v>0.1162329375046848</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>0.5375822585959787</v>
+        <v>0.5525379704355591</v>
       </c>
     </row>
     <row r="22">
@@ -1746,10 +1746,10 @@
         <v>12860000000</v>
       </c>
       <c r="H22" s="6" t="n">
-        <v>0.09891697466258816</v>
+        <v>0.1016688768048956</v>
       </c>
       <c r="I22" s="6" t="n">
-        <v>0.6364992332585669</v>
+        <v>0.6542068472404546</v>
       </c>
     </row>
     <row r="23">
@@ -1761,19 +1761,19 @@
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>22 models</t>
+          <t>19 models</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr"/>
       <c r="E23" s="7" t="inlineStr"/>
       <c r="F23" s="7" t="n">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="G23" s="8" t="n">
-        <v>47270000000</v>
+        <v>43750000000</v>
       </c>
       <c r="H23" s="9" t="n">
-        <v>0.3635007667414331</v>
+        <v>0.3457931527595452</v>
       </c>
       <c r="I23" s="9" t="n">
         <v>1</v>
@@ -1789,7 +1789,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Top 5 = 82% of class units; 5 of 15 models reach 80%. Variants merged (e.g. SPK32080/B/C, PK 41002 EH C/MH C).</t>
+          <t>Top 5 = 88% of class units; 3 of 12 models reach 80%. Variants merged (e.g. SPK32080/B/C, PK 41002 EH C/MH C).</t>
         </is>
       </c>
     </row>
@@ -1869,10 +1869,10 @@
         <v>53080000000</v>
       </c>
       <c r="H32" s="6" t="n">
-        <v>0.5342465753424658</v>
+        <v>0.5909090909090909</v>
       </c>
       <c r="I32" s="6" t="n">
-        <v>0.5342465753424658</v>
+        <v>0.5909090909090909</v>
       </c>
     </row>
     <row r="33">
@@ -1904,10 +1904,10 @@
         <v>18900000000</v>
       </c>
       <c r="H33" s="6" t="n">
-        <v>0.1643835616438356</v>
+        <v>0.1818181818181818</v>
       </c>
       <c r="I33" s="6" t="n">
-        <v>0.6986301369863014</v>
+        <v>0.7727272727272727</v>
       </c>
     </row>
     <row r="34">
@@ -1916,16 +1916,16 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>Hyva</t>
+          <t>XCMG</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>HC501X</t>
+          <t>GSQZ460.4</t>
         </is>
       </c>
       <c r="D34" s="4" t="n">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
@@ -1933,16 +1933,16 @@
         </is>
       </c>
       <c r="F34" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G34" s="5" t="n">
-        <v>4280000000</v>
+        <v>2150000000</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>0.0547945205479452</v>
+        <v>0.04545454545454546</v>
       </c>
       <c r="I34" s="6" t="n">
-        <v>0.7534246575342466</v>
+        <v>0.8181818181818181</v>
       </c>
     </row>
     <row r="35">
@@ -1951,33 +1951,33 @@
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>XCMG</t>
+          <t>Palfinger</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>GSQZ460.4</t>
+          <t>PK 76002 EH D</t>
         </is>
       </c>
       <c r="D35" s="4" t="n">
-        <v>46</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>&gt;45–50</t>
+          <t>&gt;70–75</t>
         </is>
       </c>
       <c r="F35" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G35" s="5" t="n">
-        <v>2150000000</v>
+        <v>3840000000</v>
       </c>
       <c r="H35" s="6" t="n">
-        <v>0.0410958904109589</v>
+        <v>0.0303030303030303</v>
       </c>
       <c r="I35" s="6" t="n">
-        <v>0.7945205479452055</v>
+        <v>0.8484848484848484</v>
       </c>
     </row>
     <row r="36">
@@ -1986,33 +1986,33 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>Palfinger</t>
+          <t>XCMG</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>PK 76002 EH D</t>
+          <t>GSQZ880.6</t>
         </is>
       </c>
       <c r="D36" s="4" t="n">
-        <v>71.59999999999999</v>
+        <v>88</v>
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>&gt;70–75</t>
+          <t>&gt;85–90</t>
         </is>
       </c>
       <c r="F36" s="4" t="n">
         <v>2</v>
       </c>
       <c r="G36" s="5" t="n">
-        <v>3840000000</v>
+        <v>2320000000</v>
       </c>
       <c r="H36" s="6" t="n">
-        <v>0.0273972602739726</v>
+        <v>0.0303030303030303</v>
       </c>
       <c r="I36" s="6" t="n">
-        <v>0.8219178082191781</v>
+        <v>0.8787878787878787</v>
       </c>
     </row>
     <row r="37">
@@ -2024,19 +2024,19 @@
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>10 models</t>
+          <t>7 models</t>
         </is>
       </c>
       <c r="D37" s="7" t="inlineStr"/>
       <c r="E37" s="7" t="inlineStr"/>
       <c r="F37" s="7" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="G37" s="8" t="n">
-        <v>17790000000</v>
+        <v>10910000000</v>
       </c>
       <c r="H37" s="9" t="n">
-        <v>0.1780821917808219</v>
+        <v>0.1212121212121212</v>
       </c>
       <c r="I37" s="9" t="n">
         <v>1</v>
@@ -2052,7 +2052,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Top 5 = 83% of class import value; 4 of 15 models reach 80%. Variants merged (e.g. SPK32080/B/C, PK 41002 EH C/MH C).</t>
+          <t>Top 5 = 89% of class import value; 3 of 12 models reach 80%. Variants merged (e.g. SPK32080/B/C, PK 41002 EH C/MH C).</t>
         </is>
       </c>
     </row>
@@ -2132,10 +2132,10 @@
         <v>53080000000</v>
       </c>
       <c r="H46" s="6" t="n">
-        <v>0.53063420995161</v>
+        <v>0.582054526125916</v>
       </c>
       <c r="I46" s="6" t="n">
-        <v>0.53063420995161</v>
+        <v>0.582054526125916</v>
       </c>
     </row>
     <row r="47">
@@ -2167,10 +2167,10 @@
         <v>18900000000</v>
       </c>
       <c r="H47" s="6" t="n">
-        <v>0.1889515405549896</v>
+        <v>0.2072616075931585</v>
       </c>
       <c r="I47" s="6" t="n">
-        <v>0.7195857505065997</v>
+        <v>0.7893161337190745</v>
       </c>
     </row>
     <row r="48">
@@ -2179,33 +2179,33 @@
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t>Hyva</t>
+          <t>Palfinger</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>HC501X</t>
+          <t>PK 76002 EH D</t>
         </is>
       </c>
       <c r="D48" s="4" t="n">
-        <v>50</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t>&gt;45–50</t>
+          <t>&gt;70–75</t>
         </is>
       </c>
       <c r="F48" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G48" s="5" t="n">
-        <v>4280000000</v>
+        <v>3840000000</v>
       </c>
       <c r="H48" s="6" t="n">
-        <v>0.04275678485336782</v>
+        <v>0.04205246414423664</v>
       </c>
       <c r="I48" s="6" t="n">
-        <v>0.7623425353599675</v>
+        <v>0.8313685978633112</v>
       </c>
     </row>
     <row r="49">
@@ -2214,33 +2214,33 @@
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>Palfinger</t>
+          <t>Hiab</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>PK 76002 EH D</t>
+          <t>X-HIPRO B58</t>
         </is>
       </c>
       <c r="D49" s="4" t="n">
-        <v>71.59999999999999</v>
+        <v>50.93</v>
       </c>
       <c r="E49" s="4" t="inlineStr">
         <is>
-          <t>&gt;70–75</t>
+          <t>&gt;50–55</t>
         </is>
       </c>
       <c r="F49" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G49" s="5" t="n">
-        <v>3840000000</v>
+        <v>2820000000</v>
       </c>
       <c r="H49" s="6" t="n">
-        <v>0.0383374324673976</v>
+        <v>0.03096974206637752</v>
       </c>
       <c r="I49" s="6" t="n">
-        <v>0.8006799678273652</v>
+        <v>0.8623383399296887</v>
       </c>
     </row>
     <row r="50">
@@ -2249,33 +2249,33 @@
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t>Hyva</t>
+          <t>XCMG</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>HB660R</t>
+          <t>GSQZ880.6</t>
         </is>
       </c>
       <c r="D50" s="4" t="n">
-        <v>60</v>
+        <v>88</v>
       </c>
       <c r="E50" s="4" t="inlineStr">
         <is>
-          <t>&gt;55–60</t>
+          <t>&gt;85–90</t>
         </is>
       </c>
       <c r="F50" s="4" t="n">
         <v>2</v>
       </c>
       <c r="G50" s="5" t="n">
-        <v>3090000000</v>
+        <v>2320000000</v>
       </c>
       <c r="H50" s="6" t="n">
-        <v>0.03090434872529247</v>
+        <v>0.0254893394149508</v>
       </c>
       <c r="I50" s="6" t="n">
-        <v>0.8315843165526576</v>
+        <v>0.8878276793446395</v>
       </c>
     </row>
     <row r="51">
@@ -2287,19 +2287,19 @@
       </c>
       <c r="C51" s="7" t="inlineStr">
         <is>
-          <t>10 models</t>
+          <t>7 models</t>
         </is>
       </c>
       <c r="D51" s="7" t="inlineStr"/>
       <c r="E51" s="7" t="inlineStr"/>
       <c r="F51" s="7" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="G51" s="8" t="n">
-        <v>16850000000</v>
+        <v>10230000000</v>
       </c>
       <c r="H51" s="9" t="n">
-        <v>0.1684156834473425</v>
+        <v>0.1121723206553603</v>
       </c>
       <c r="I51" s="9" t="n">
         <v>1</v>
@@ -2317,7 +2317,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2404,7 +2404,7 @@
         </is>
       </c>
       <c r="B5" s="14" t="n">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C5" s="13" t="inlineStr">
         <is>
@@ -2450,12 +2450,12 @@
         </is>
       </c>
       <c r="B7" s="14" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="C7" s="13" t="inlineStr">
         <is>
           <t>SPK42502 (42.5 tm)
-18 units · 69% of class
+18 units · 78% of class
 Rp 790.000.000 per unit</t>
         </is>
       </c>
@@ -2511,12 +2511,7 @@
           <t>Amco Veba</t>
         </is>
       </c>
-      <c r="G12" s="11" t="inlineStr">
-        <is>
-          <t>Hyva</t>
-        </is>
-      </c>
-      <c r="H12" s="12" t="inlineStr">
+      <c r="G12" s="12" t="inlineStr">
         <is>
           <t>F.lli Ferrari</t>
         </is>
@@ -2529,7 +2524,7 @@
         </is>
       </c>
       <c r="B13" s="14" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="C13" s="14" t="n"/>
       <c r="D13" s="14" t="n"/>
@@ -2537,12 +2532,11 @@
       <c r="F13" s="13" t="inlineStr">
         <is>
           <t>V950 (45.9 tm)
-12 units · 55% of class
+12 units · 67% of class
 Rp 1.880.000.000 per unit</t>
         </is>
       </c>
-      <c r="G13" s="14" t="n"/>
-      <c r="H13" s="15" t="inlineStr">
+      <c r="G13" s="15" t="inlineStr">
         <is>
           <t>FBR450R A4 (45.5 tm) · Rp 1.780.000.000</t>
         </is>
@@ -2567,8 +2561,7 @@
       </c>
       <c r="E14" s="14" t="n"/>
       <c r="F14" s="14" t="n"/>
-      <c r="G14" s="14" t="n"/>
-      <c r="H14" s="15" t="inlineStr">
+      <c r="G14" s="15" t="inlineStr">
         <is>
           <t>No Ferrari model</t>
         </is>
@@ -2580,23 +2573,18 @@
           <t>&gt;55–60</t>
         </is>
       </c>
-      <c r="B15" s="14" t="n">
-        <v>3</v>
+      <c r="B15" s="14" t="inlineStr">
+        <is>
+          <t>No imports</t>
+        </is>
       </c>
       <c r="C15" s="14" t="n"/>
       <c r="D15" s="14" t="n"/>
       <c r="E15" s="14" t="n"/>
       <c r="F15" s="14" t="n"/>
-      <c r="G15" s="13" t="inlineStr">
-        <is>
-          <t>HB660R (60 tm)
-2 units · 67% of class
-Rp 1.840.000.000 per unit</t>
-        </is>
-      </c>
-      <c r="H15" s="15" t="inlineStr">
-        <is>
-          <t>FBR660R A4 (58.8 tm) · Rp 2.660.000.000</t>
+      <c r="G15" s="15" t="inlineStr">
+        <is>
+          <t>FBR600R A4 (57.4 tm) · Rp 2.620.000.000</t>
         </is>
       </c>
     </row>
@@ -2619,8 +2607,7 @@
       <c r="D16" s="14" t="n"/>
       <c r="E16" s="14" t="n"/>
       <c r="F16" s="14" t="n"/>
-      <c r="G16" s="14" t="n"/>
-      <c r="H16" s="15" t="inlineStr">
+      <c r="G16" s="15" t="inlineStr">
         <is>
           <t>9661C (63.2 tm) · price not yet known</t>
         </is>
@@ -2645,8 +2632,7 @@
       </c>
       <c r="E17" s="14" t="n"/>
       <c r="F17" s="14" t="n"/>
-      <c r="G17" s="14" t="n"/>
-      <c r="H17" s="15" t="inlineStr">
+      <c r="G17" s="15" t="inlineStr">
         <is>
           <t>990R (74 tm) · price not yet known</t>
         </is>
@@ -2671,8 +2657,7 @@
       </c>
       <c r="E18" s="14" t="n"/>
       <c r="F18" s="14" t="n"/>
-      <c r="G18" s="14" t="n"/>
-      <c r="H18" s="15" t="inlineStr">
+      <c r="G18" s="15" t="inlineStr">
         <is>
           <t>No Ferrari model</t>
         </is>
@@ -2697,8 +2682,7 @@
         </is>
       </c>
       <c r="F19" s="14" t="n"/>
-      <c r="G19" s="14" t="n"/>
-      <c r="H19" s="15" t="inlineStr">
+      <c r="G19" s="15" t="inlineStr">
         <is>
           <t>No Ferrari model</t>
         </is>

</xml_diff>